<commit_message>
Penambahan API report.form.dataList.master.businessDocumentType.getAll, report.form.dataList.master.businessDocumentType.getTransactionDocument, dan report.form.dataList.master.businessDocumentType.getMasterData. Perubahan API report.form.dataList.master.getBank -> report.form.dataList.master.bank.getAll dan report.form.dataList.master.getBankAccount -> report.form.dataList.master.bankAccount.getAll
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
+++ b/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
@@ -94,15 +94,6 @@
     <t>Sales Quotation Form</t>
   </si>
   <si>
-    <t>Sales Quote Cancelation Form</t>
-  </si>
-  <si>
-    <t>Sales Quote Revision Form</t>
-  </si>
-  <si>
-    <t>Sales Quote Revision Cancelation Form</t>
-  </si>
-  <si>
     <t>Sales Order Form</t>
   </si>
   <si>
@@ -479,6 +470,15 @@
   </si>
   <si>
     <t>Customer Master Data</t>
+  </si>
+  <si>
+    <t>Sales Quotation Cancelation Form</t>
+  </si>
+  <si>
+    <t>Sales Quotation Revision Form</t>
+  </si>
+  <si>
+    <t>Sales Quotation Revision Cancelation Form</t>
   </si>
 </sst>
 </file>
@@ -964,7 +964,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>2</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>26</v>
+        <v>152</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="6" t="b">
@@ -1025,12 +1025,12 @@
 "'signTransactionDocument', ", IF(EXACT($D5, ""), "null", CONCATENATE("'", SUBSTITUTE($D5, "'", "\'"), "'")), "::varchar,",
 "'paymenStatus', ", IF(EXACT($E5, ""), "null", CONCATENATE("'", SUBSTITUTE($E5, "'", "\'"), "'")), "::varchar",
 ")))::varchar;")</f>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quote Cancelation Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quotation Cancelation Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>153</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6" t="b">
@@ -1039,12 +1039,12 @@
       <c r="E6" s="5"/>
       <c r="G6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quote Revision Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quotation Revision Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
-        <v>28</v>
+        <v>154</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="6" t="b">
@@ -1053,12 +1053,12 @@
       <c r="E7" s="5"/>
       <c r="G7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quote Revision Cancelation Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quotation Revision Cancelation Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="6" t="b">
@@ -1072,7 +1072,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="6" t="b">
@@ -1086,7 +1086,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="6" t="b">
@@ -1100,7 +1100,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="6" t="b">
@@ -1114,7 +1114,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="6" t="b">
@@ -1128,7 +1128,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="6" t="b">
@@ -1142,7 +1142,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="6" t="b">
@@ -1156,7 +1156,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="6" t="b">
@@ -1186,7 +1186,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="6" t="b">
@@ -1200,7 +1200,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="6" t="b">
@@ -1214,7 +1214,7 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="6" t="b">
@@ -1244,7 +1244,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="6" t="b">
@@ -1258,7 +1258,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="6" t="b">
@@ -1272,7 +1272,7 @@
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="6" t="b">
@@ -1286,7 +1286,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="6" t="b">
@@ -1300,7 +1300,7 @@
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="6" t="b">
@@ -1314,7 +1314,7 @@
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="6" t="b">
@@ -1328,7 +1328,7 @@
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="6" t="b">
@@ -1342,7 +1342,7 @@
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="6" t="b">
@@ -1356,7 +1356,7 @@
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="6" t="b">
@@ -1370,7 +1370,7 @@
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="6" t="b">
@@ -1384,7 +1384,7 @@
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="6" t="b">
@@ -1398,7 +1398,7 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="6" t="b">
@@ -1412,7 +1412,7 @@
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="b">
@@ -1426,7 +1426,7 @@
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="b">
@@ -1440,7 +1440,7 @@
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="6" t="b">
@@ -1454,7 +1454,7 @@
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="6" t="b">
@@ -1468,7 +1468,7 @@
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="6" t="b">
@@ -1482,7 +1482,7 @@
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B38" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="6" t="b">
@@ -1496,7 +1496,7 @@
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="6" t="b">
@@ -1526,7 +1526,7 @@
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="6" t="b">
@@ -1540,7 +1540,7 @@
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="6" t="b">
@@ -1554,7 +1554,7 @@
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="6" t="b">
@@ -1584,7 +1584,7 @@
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="6" t="b">
@@ -1598,7 +1598,7 @@
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="6" t="b">
@@ -1612,7 +1612,7 @@
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="6" t="b">
@@ -1642,7 +1642,7 @@
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B49" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="6" t="b">
@@ -1656,7 +1656,7 @@
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B50" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="6" t="b">
@@ -1670,7 +1670,7 @@
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B51" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="6" t="b">
@@ -1700,7 +1700,7 @@
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B53" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="6" t="b">
@@ -1714,7 +1714,7 @@
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B54" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="6" t="b">
@@ -1728,7 +1728,7 @@
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B55" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="6" t="b">
@@ -1758,7 +1758,7 @@
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B57" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="6" t="b">
@@ -1772,7 +1772,7 @@
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B58" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="6" t="b">
@@ -1786,7 +1786,7 @@
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B59" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C59" s="5"/>
       <c r="D59" s="6" t="b">
@@ -1818,7 +1818,7 @@
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B61" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="6" t="b">
@@ -1832,7 +1832,7 @@
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B62" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C62" s="5"/>
       <c r="D62" s="6" t="b">
@@ -1846,7 +1846,7 @@
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B63" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C63" s="5"/>
       <c r="D63" s="6" t="b">
@@ -1876,7 +1876,7 @@
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B65" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C65" s="5"/>
       <c r="D65" s="6" t="b">
@@ -1890,7 +1890,7 @@
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B66" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="6" t="b">
@@ -1904,7 +1904,7 @@
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B67" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C67" s="5"/>
       <c r="D67" s="6" t="b">
@@ -1936,7 +1936,7 @@
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B69" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C69" s="5"/>
       <c r="D69" s="6" t="b">
@@ -1965,7 +1965,7 @@
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B70" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C70" s="5"/>
       <c r="D70" s="6" t="b">
@@ -1979,7 +1979,7 @@
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B71" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C71" s="5"/>
       <c r="D71" s="6" t="b">
@@ -2009,7 +2009,7 @@
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B73" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C73" s="5"/>
       <c r="D73" s="6" t="b">
@@ -2023,7 +2023,7 @@
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B74" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C74" s="5"/>
       <c r="D74" s="6" t="b">
@@ -2037,7 +2037,7 @@
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B75" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="6" t="b">
@@ -2051,7 +2051,7 @@
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B76" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C76" s="5"/>
       <c r="D76" s="6" t="b">
@@ -2065,7 +2065,7 @@
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B77" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C77" s="5"/>
       <c r="D77" s="6" t="b">
@@ -2079,7 +2079,7 @@
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B78" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C78" s="5"/>
       <c r="D78" s="6" t="b">
@@ -2093,7 +2093,7 @@
     </row>
     <row r="79" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B79" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C79" s="5"/>
       <c r="D79" s="6" t="b">
@@ -2123,7 +2123,7 @@
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B81" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="6" t="b">
@@ -2137,7 +2137,7 @@
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B82" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C82" s="5"/>
       <c r="D82" s="6" t="b">
@@ -2151,7 +2151,7 @@
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B83" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="6" t="b">
@@ -2181,7 +2181,7 @@
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B85" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C85" s="5"/>
       <c r="D85" s="6" t="b">
@@ -2195,7 +2195,7 @@
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B86" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C86" s="5"/>
       <c r="D86" s="6" t="b">
@@ -2209,7 +2209,7 @@
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B87" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C87" s="5"/>
       <c r="D87" s="6" t="b">
@@ -2239,7 +2239,7 @@
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B89" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C89" s="5"/>
       <c r="D89" s="6" t="b">
@@ -2253,7 +2253,7 @@
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B90" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C90" s="5"/>
       <c r="D90" s="6" t="b">
@@ -2267,7 +2267,7 @@
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B91" s="4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C91" s="5"/>
       <c r="D91" s="6" t="b">
@@ -2297,7 +2297,7 @@
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B93" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C93" s="5"/>
       <c r="D93" s="6" t="b">
@@ -2311,7 +2311,7 @@
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B94" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C94" s="5"/>
       <c r="D94" s="6" t="b">
@@ -2325,7 +2325,7 @@
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B95" s="4" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C95" s="5"/>
       <c r="D95" s="6" t="b">
@@ -2339,7 +2339,7 @@
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B96" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C96" s="5"/>
       <c r="D96" s="6" t="b">
@@ -2353,7 +2353,7 @@
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B97" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C97" s="5"/>
       <c r="D97" s="6" t="b">
@@ -2367,7 +2367,7 @@
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B98" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C98" s="5"/>
       <c r="D98" s="6" t="b">
@@ -2381,7 +2381,7 @@
     </row>
     <row r="99" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B99" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C99" s="5"/>
       <c r="D99" s="6" t="b">
@@ -2411,7 +2411,7 @@
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B101" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C101" s="5"/>
       <c r="D101" s="6" t="b">
@@ -2425,7 +2425,7 @@
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B102" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C102" s="5"/>
       <c r="D102" s="6" t="b">
@@ -2439,7 +2439,7 @@
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B103" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C103" s="5"/>
       <c r="D103" s="6" t="b">
@@ -2453,7 +2453,7 @@
     </row>
     <row r="104" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B104" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C104" s="5"/>
       <c r="D104" s="6" t="b">
@@ -2467,7 +2467,7 @@
     </row>
     <row r="105" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B105" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="6" t="b">
@@ -2481,7 +2481,7 @@
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B106" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C106" s="5"/>
       <c r="D106" s="6" t="b">
@@ -2495,7 +2495,7 @@
     </row>
     <row r="107" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B107" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C107" s="5"/>
       <c r="D107" s="6" t="b">
@@ -2509,7 +2509,7 @@
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B108" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C108" s="5"/>
       <c r="D108" s="6" t="b">
@@ -2523,7 +2523,7 @@
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B109" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C109" s="5"/>
       <c r="D109" s="6" t="b">
@@ -2537,7 +2537,7 @@
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B110" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C110" s="5"/>
       <c r="D110" s="6" t="b">
@@ -2551,7 +2551,7 @@
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B111" s="4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C111" s="5"/>
       <c r="D111" s="6" t="b">
@@ -2565,7 +2565,7 @@
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B112" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C112" s="5"/>
       <c r="D112" s="6" t="b">
@@ -2579,7 +2579,7 @@
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B113" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C113" s="5"/>
       <c r="D113" s="6" t="b">
@@ -2593,7 +2593,7 @@
     </row>
     <row r="114" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B114" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C114" s="5"/>
       <c r="D114" s="6" t="b">
@@ -2607,7 +2607,7 @@
     </row>
     <row r="115" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B115" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C115" s="5"/>
       <c r="D115" s="6" t="b">
@@ -2621,7 +2621,7 @@
     </row>
     <row r="116" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B116" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C116" s="5"/>
       <c r="D116" s="6" t="b">
@@ -2635,7 +2635,7 @@
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B117" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C117" s="5"/>
       <c r="D117" s="6" t="b">
@@ -2649,7 +2649,7 @@
     </row>
     <row r="118" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B118" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C118" s="5"/>
       <c r="D118" s="6" t="b">
@@ -2663,7 +2663,7 @@
     </row>
     <row r="119" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B119" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C119" s="5"/>
       <c r="D119" s="6" t="b">
@@ -2677,7 +2677,7 @@
     </row>
     <row r="120" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B120" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C120" s="5"/>
       <c r="D120" s="6" t="b">
@@ -2691,7 +2691,7 @@
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B121" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C121" s="5"/>
       <c r="D121" s="6" t="b">
@@ -2705,7 +2705,7 @@
     </row>
     <row r="122" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B122" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C122" s="5"/>
       <c r="D122" s="6" t="b">
@@ -2719,7 +2719,7 @@
     </row>
     <row r="123" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B123" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C123" s="5"/>
       <c r="D123" s="6" t="b">
@@ -2749,7 +2749,7 @@
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B125" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C125" s="5"/>
       <c r="D125" s="6" t="b">
@@ -2763,7 +2763,7 @@
     </row>
     <row r="126" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B126" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C126" s="5"/>
       <c r="D126" s="6" t="b">
@@ -2777,7 +2777,7 @@
     </row>
     <row r="127" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B127" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C127" s="5"/>
       <c r="D127" s="6" t="b">
@@ -2807,7 +2807,7 @@
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B129" s="4" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C129" s="5"/>
       <c r="D129" s="6" t="b">
@@ -2821,7 +2821,7 @@
     </row>
     <row r="130" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B130" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C130" s="5"/>
       <c r="D130" s="6" t="b">
@@ -2835,7 +2835,7 @@
     </row>
     <row r="131" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B131" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C131" s="5"/>
       <c r="D131" s="6" t="b">
@@ -2865,7 +2865,7 @@
     </row>
     <row r="133" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B133" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C133" s="5"/>
       <c r="D133" s="6" t="b">
@@ -2894,7 +2894,7 @@
     </row>
     <row r="134" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B134" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C134" s="5"/>
       <c r="D134" s="6" t="b">
@@ -2908,7 +2908,7 @@
     </row>
     <row r="135" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B135" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C135" s="5"/>
       <c r="D135" s="6" t="b">
@@ -2938,7 +2938,7 @@
     </row>
     <row r="137" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B137" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C137" s="5"/>
       <c r="D137" s="6" t="b">
@@ -2952,7 +2952,7 @@
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B138" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C138" s="5"/>
       <c r="D138" s="6" t="b">
@@ -2966,7 +2966,7 @@
     </row>
     <row r="139" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B139" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C139" s="5"/>
       <c r="D139" s="6" t="b">
@@ -2996,7 +2996,7 @@
     </row>
     <row r="141" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B141" s="4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C141" s="5"/>
       <c r="D141" s="6" t="b">
@@ -3010,7 +3010,7 @@
     </row>
     <row r="142" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B142" s="4" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C142" s="5"/>
       <c r="D142" s="6" t="b">
@@ -3024,7 +3024,7 @@
     </row>
     <row r="143" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B143" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C143" s="5"/>
       <c r="D143" s="6" t="b">
@@ -3054,7 +3054,7 @@
     </row>
     <row r="145" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B145" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C145" s="5"/>
       <c r="D145" s="6" t="b">
@@ -3068,7 +3068,7 @@
     </row>
     <row r="146" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B146" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C146" s="5"/>
       <c r="D146" s="6" t="b">
@@ -3082,7 +3082,7 @@
     </row>
     <row r="147" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B147" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C147" s="5"/>
       <c r="D147" s="6" t="b">
@@ -3096,7 +3096,7 @@
     </row>
     <row r="148" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B148" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C148" s="5"/>
       <c r="D148" s="6" t="b">
@@ -3110,7 +3110,7 @@
     </row>
     <row r="149" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B149" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C149" s="5"/>
       <c r="D149" s="6" t="b">
@@ -3124,7 +3124,7 @@
     </row>
     <row r="150" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B150" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C150" s="5"/>
       <c r="D150" s="6" t="b">
@@ -3138,7 +3138,7 @@
     </row>
     <row r="151" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B151" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C151" s="5"/>
       <c r="D151" s="6" t="b">
@@ -3152,7 +3152,7 @@
     </row>
     <row r="152" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B152" s="8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C152" s="9"/>
       <c r="D152" s="10" t="b">
@@ -3166,7 +3166,7 @@
     </row>
     <row r="153" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B153" s="8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C153" s="9"/>
       <c r="D153" s="10" t="b">
@@ -3180,7 +3180,7 @@
     </row>
     <row r="154" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B154" s="8" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C154" s="9"/>
       <c r="D154" s="10" t="b">

</xml_diff>

<commit_message>
Update Pertanggal 4 September 2026 Malam
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
+++ b/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
@@ -974,7 +974,9 @@
       <c r="B4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="5"/>
+      <c r="C4" s="5">
+        <v>3000000000136</v>
+      </c>
       <c r="D4" s="6" t="b">
         <v>1</v>
       </c>
@@ -996,7 +998,7 @@
 "'signTransactionDocument', ", IF(EXACT($D4, ""), "null", CONCATENATE("'", SUBSTITUTE($D4, "'", "\'"), "'")), "::varchar,",
 "'paymenStatus', ", IF(EXACT($E4, ""), "null", CONCATENATE("'", SUBSTITUTE($E4, "'", "\'"), "'")), "::varchar",
 ")))::varchar;")</f>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quotation Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Quotation Form'::varchar,'table_RefID', '3000000000136'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
@@ -1060,14 +1062,16 @@
       <c r="B8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="5"/>
+      <c r="C8" s="5">
+        <v>3000000000129</v>
+      </c>
       <c r="D8" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E8" s="5"/>
       <c r="G8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Order Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Order Form'::varchar,'table_RefID', '3000000000129'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
@@ -1116,14 +1120,16 @@
       <c r="B12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="5"/>
+      <c r="C12" s="5">
+        <v>3000000000131</v>
+      </c>
       <c r="D12" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E12" s="5"/>
       <c r="G12" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Contract Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Contract Form'::varchar,'table_RefID', '3000000000131'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
@@ -1172,7 +1178,9 @@
       <c r="B16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="5"/>
+      <c r="C16" s="5">
+        <v>3000000000046</v>
+      </c>
       <c r="D16" s="6" t="b">
         <v>1</v>
       </c>
@@ -1181,7 +1189,7 @@
       </c>
       <c r="G16" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Form'::varchar,'table_RefID', '3000000000046'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
@@ -1230,7 +1238,9 @@
       <c r="B20" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="5"/>
+      <c r="C20" s="5">
+        <v>3000000000110</v>
+      </c>
       <c r="D20" s="6" t="b">
         <v>1</v>
       </c>
@@ -1239,7 +1249,7 @@
       </c>
       <c r="G20" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Form'::varchar,'table_RefID', '3000000000110'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
@@ -1288,14 +1298,16 @@
       <c r="B24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="5">
+        <v>3000000000143</v>
+      </c>
       <c r="D24" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E24" s="5"/>
       <c r="G24" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Item Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Item Form'::varchar,'table_RefID', '3000000000143'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
@@ -1344,14 +1356,16 @@
       <c r="B28" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="5"/>
+      <c r="C28" s="5">
+        <v>3000000000158</v>
+      </c>
       <c r="D28" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E28" s="5"/>
       <c r="G28" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Item Work Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Project Section Item Work Form'::varchar,'table_RefID', '3000000000158'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
@@ -1512,7 +1526,9 @@
       <c r="B40" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C40" s="5"/>
+      <c r="C40" s="5">
+        <v>3000000000103</v>
+      </c>
       <c r="D40" s="6" t="b">
         <v>1</v>
       </c>
@@ -1521,7 +1537,7 @@
       </c>
       <c r="G40" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Budget Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Budget Form'::varchar,'table_RefID', '3000000000103'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
@@ -1570,7 +1586,9 @@
       <c r="B44" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="5"/>
+      <c r="C44" s="5">
+        <v>3000000000083</v>
+      </c>
       <c r="D44" s="6" t="b">
         <v>1</v>
       </c>
@@ -1579,7 +1597,7 @@
       </c>
       <c r="G44" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Purchase Requisition Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Purchase Requisition Form'::varchar,'table_RefID', '3000000000083'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.2">
@@ -1628,7 +1646,9 @@
       <c r="B48" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C48" s="5"/>
+      <c r="C48" s="5">
+        <v>3000000000085</v>
+      </c>
       <c r="D48" s="6" t="b">
         <v>1</v>
       </c>
@@ -1637,7 +1657,7 @@
       </c>
       <c r="G48" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Purchase Order Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Purchase Order Form'::varchar,'table_RefID', '3000000000085'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.2">
@@ -1686,7 +1706,9 @@
       <c r="B52" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="5"/>
+      <c r="C52" s="5">
+        <v>3000000000211</v>
+      </c>
       <c r="D52" s="6" t="b">
         <v>1</v>
       </c>
@@ -1695,7 +1717,7 @@
       </c>
       <c r="G52" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Payment Instruction Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Payment Instruction Form'::varchar,'table_RefID', '3000000000211'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.2">
@@ -1744,7 +1766,9 @@
       <c r="B56" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C56" s="5"/>
+      <c r="C56" s="5">
+        <v>3000000000192</v>
+      </c>
       <c r="D56" s="6" t="b">
         <v>1</v>
       </c>
@@ -1753,7 +1777,7 @@
       </c>
       <c r="G56" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Cash Disbursement Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Cash Disbursement Form'::varchar,'table_RefID', '3000000000192'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.2">
@@ -2053,14 +2077,16 @@
       <c r="B76" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C76" s="5"/>
+      <c r="C76" s="5">
+        <v>3000000000048</v>
+      </c>
       <c r="D76" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E76" s="5"/>
       <c r="G76" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Timesheet Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Timesheet Form'::varchar,'table_RefID', '3000000000048'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.2">
@@ -2109,7 +2135,9 @@
       <c r="B80" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C80" s="5"/>
+      <c r="C80" s="5">
+        <v>3000000000180</v>
+      </c>
       <c r="D80" s="6" t="b">
         <v>1</v>
       </c>
@@ -2118,7 +2146,7 @@
       </c>
       <c r="G80" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Delivery Order Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Delivery Order Form'::varchar,'table_RefID', '3000000000180'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.2">
@@ -2167,7 +2195,9 @@
       <c r="B84" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C84" s="5"/>
+      <c r="C84" s="5">
+        <v>3000000000176</v>
+      </c>
       <c r="D84" s="6" t="b">
         <v>1</v>
       </c>
@@ -2176,7 +2206,7 @@
       </c>
       <c r="G84" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Warehouse Inbound Order Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Warehouse Inbound Order Form'::varchar,'table_RefID', '3000000000176'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.2">
@@ -2225,7 +2255,9 @@
       <c r="B88" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C88" s="5"/>
+      <c r="C88" s="5">
+        <v>3000000000178</v>
+      </c>
       <c r="D88" s="6" t="b">
         <v>1</v>
       </c>
@@ -2234,7 +2266,7 @@
       </c>
       <c r="G88" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Warehouse Outbound Order Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Warehouse Outbound Order Form'::varchar,'table_RefID', '3000000000178'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.2">
@@ -2283,7 +2315,9 @@
       <c r="B92" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C92" s="5"/>
+      <c r="C92" s="5">
+        <v>3000000000242</v>
+      </c>
       <c r="D92" s="6" t="b">
         <v>1</v>
       </c>
@@ -2292,7 +2326,7 @@
       </c>
       <c r="G92" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Credit Note Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Credit Note Form'::varchar,'table_RefID', '3000000000242'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.2">
@@ -2341,14 +2375,16 @@
       <c r="B96" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C96" s="5"/>
+      <c r="C96" s="5">
+        <v>3000000000240</v>
+      </c>
       <c r="D96" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E96" s="5"/>
       <c r="G96" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Debit Note Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Debit Note Form'::varchar,'table_RefID', '3000000000240'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.2">
@@ -2397,7 +2433,9 @@
       <c r="B100" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C100" s="5"/>
+      <c r="C100" s="5">
+        <v>3000000000203</v>
+      </c>
       <c r="D100" s="6" t="b">
         <v>1</v>
       </c>
@@ -2406,7 +2444,7 @@
       </c>
       <c r="G100" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Advance Settlement Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Advance Settlement Form'::varchar,'table_RefID', '3000000000203'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.2">
@@ -2455,14 +2493,16 @@
       <c r="B104" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C104" s="5"/>
+      <c r="C104" s="5">
+        <v>3000000000244</v>
+      </c>
       <c r="D104" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E104" s="5"/>
       <c r="G104" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Invoice Request Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Invoice Request Form'::varchar,'table_RefID', '3000000000244'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="105" spans="2:7" x14ac:dyDescent="0.2">
@@ -2511,14 +2551,16 @@
       <c r="B108" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C108" s="5"/>
+      <c r="C108" s="5">
+        <v>3000000000138</v>
+      </c>
       <c r="D108" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E108" s="5"/>
       <c r="G108" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Invoice Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Sales Invoice Form'::varchar,'table_RefID', '3000000000138'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.2">
@@ -2567,14 +2609,16 @@
       <c r="B112" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C112" s="5"/>
+      <c r="C112" s="5">
+        <v>3000000000248</v>
+      </c>
       <c r="D112" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E112" s="5"/>
       <c r="G112" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Order Picking Requisition Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Order Picking Requisition Form'::varchar,'table_RefID', '3000000000248'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.2">
@@ -2623,14 +2667,16 @@
       <c r="B116" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C116" s="5"/>
+      <c r="C116" s="5">
+        <v>3000000000250</v>
+      </c>
       <c r="D116" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E116" s="5"/>
       <c r="G116" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Order Picking Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Order Picking Form'::varchar,'table_RefID', '3000000000250'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.2">
@@ -2679,14 +2725,16 @@
       <c r="B120" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="C120" s="5"/>
+      <c r="C120" s="5">
+        <v>3000000000262</v>
+      </c>
       <c r="D120" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E120" s="5"/>
       <c r="G120" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Material Service Requisition Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Material Service Requisition Form'::varchar,'table_RefID', '3000000000262'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.2">
@@ -2735,7 +2783,9 @@
       <c r="B124" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C124" s="5"/>
+      <c r="C124" s="5">
+        <v>3000000000078</v>
+      </c>
       <c r="D124" s="6" t="b">
         <v>1</v>
       </c>
@@ -2744,7 +2794,7 @@
       </c>
       <c r="G124" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Person Business Trip Settlement Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Person Business Trip Settlement Form'::varchar,'table_RefID', '3000000000078'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.2">
@@ -2793,7 +2843,9 @@
       <c r="B128" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C128" s="5"/>
+      <c r="C128" s="5">
+        <v>3000000000288</v>
+      </c>
       <c r="D128" s="6" t="b">
         <v>1</v>
       </c>
@@ -2802,7 +2854,7 @@
       </c>
       <c r="G128" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Reimbursement Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Reimbursement Form'::varchar,'table_RefID', '3000000000288'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '1'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.2">
@@ -2851,7 +2903,9 @@
       <c r="B132" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C132" s="5"/>
+      <c r="C132" s="5">
+        <v>3000000000290</v>
+      </c>
       <c r="D132" s="6" t="b">
         <v>1</v>
       </c>
@@ -2860,7 +2914,7 @@
       </c>
       <c r="G132" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Cash Receipt Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Cash Receipt Form'::varchar,'table_RefID', '3000000000290'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="133" spans="2:7" x14ac:dyDescent="0.2">
@@ -2924,7 +2978,9 @@
       <c r="B136" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C136" s="5"/>
+      <c r="C136" s="5">
+        <v>3000000000293</v>
+      </c>
       <c r="D136" s="6" t="b">
         <v>1</v>
       </c>
@@ -2933,7 +2989,7 @@
       </c>
       <c r="G136" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Loan Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Loan Form'::varchar,'table_RefID', '3000000000293'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="137" spans="2:7" x14ac:dyDescent="0.2">
@@ -2982,7 +3038,9 @@
       <c r="B140" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C140" s="5"/>
+      <c r="C140" s="5">
+        <v>3000000000295</v>
+      </c>
       <c r="D140" s="6" t="b">
         <v>1</v>
       </c>
@@ -2991,7 +3049,7 @@
       </c>
       <c r="G140" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Loan Settlement Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Loan Settlement Form'::varchar,'table_RefID', '3000000000295'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="141" spans="2:7" x14ac:dyDescent="0.2">
@@ -3040,7 +3098,9 @@
       <c r="B144" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C144" s="5"/>
+      <c r="C144" s="5">
+        <v>3000000000068</v>
+      </c>
       <c r="D144" s="6" t="b">
         <v>1</v>
       </c>
@@ -3049,7 +3109,7 @@
       </c>
       <c r="G144" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Journal Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Journal Form'::varchar,'table_RefID', '3000000000068'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '0'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="145" spans="2:7" x14ac:dyDescent="0.2">
@@ -3098,14 +3158,16 @@
       <c r="B148" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C148" s="5"/>
+      <c r="C148" s="5">
+        <v>3000000000069</v>
+      </c>
       <c r="D148" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E148" s="5"/>
       <c r="G148" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Journal Detail Form'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Journal Detail Form'::varchar,'table_RefID', '3000000000069'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="149" spans="2:7" x14ac:dyDescent="0.2">
@@ -3154,42 +3216,48 @@
       <c r="B152" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C152" s="9"/>
+      <c r="C152" s="9">
+        <v>3000000000088</v>
+      </c>
       <c r="D152" s="10" t="b">
         <v>0</v>
       </c>
       <c r="E152" s="9"/>
       <c r="G152" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Product Master Data'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Product Master Data'::varchar,'table_RefID', '3000000000088'::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="153" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B153" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C153" s="9"/>
+      <c r="C153" s="9">
+        <v>3000000000126</v>
+      </c>
       <c r="D153" s="10" t="b">
         <v>0</v>
       </c>
       <c r="E153" s="9"/>
       <c r="G153" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Supplier Master Data'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Supplier Master Data'::varchar,'table_RefID', '3000000000126'::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="154" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B154" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="C154" s="9"/>
+      <c r="C154" s="9">
+        <v>3000000000125</v>
+      </c>
       <c r="D154" s="10" t="b">
         <v>0</v>
       </c>
       <c r="E154" s="9"/>
       <c r="G154" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Customer Master Data'::varchar,'table_RefID', null::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Customer Master Data'::varchar,'table_RefID', '3000000000125'::varchar,'signTransactionDocument', 'FALSE'::varchar,'paymenStatus', null::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="155" spans="2:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update Pertanggal 9 September 2026 Pagi
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
+++ b/Documentation/Documents/SQL Generator/Data Initial/Master.TblBusinessDocumentType.xlsx
@@ -2784,7 +2784,7 @@
         <v>19</v>
       </c>
       <c r="C124" s="5">
-        <v>3000000000078</v>
+        <v>3000000000274</v>
       </c>
       <c r="D124" s="6" t="b">
         <v>1</v>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="G124" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Person Business Trip Settlement Form'::varchar,'table_RefID', '3000000000078'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'name', 'Person Business Trip Settlement Form'::varchar,'table_RefID', '3000000000274'::varchar,'signTransactionDocument', 'TRUE'::varchar,'paymenStatus', '2'::varchar)))::varchar;</v>
       </c>
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.2">

</xml_diff>